<commit_message>
Painel da clinica: bater o limite exato deixa o cartao amarelo (nao verde); telas, mockups, OG e heroi refeitos
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-medicos/17-painel-da-clinica.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-medicos/17-painel-da-clinica.xlsx
@@ -1643,7 +1643,7 @@
       </c>
       <c r="E20" s="19" t="str">
         <f>Dados!F9</f>
-        <v>No alvo</v>
+        <v>Perto</v>
       </c>
       <c r="F20" s="24">
         <f>IF(Config!$B$8&lt;=1,"—",IF(INDEX(Histórico!$F$5:$F$16,Config!$B$8-1)="","—",INDEX(Histórico!$F$5:$F$16,Config!$B$8-1)))</f>
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="F5" s="19" t="str">
-        <f>IF(OR(B5="",C5=""),"Informativo",IF(D5="Menor é melhor",IF(B5&lt;=C5,"No alvo",IF(B5&lt;=C5*1.1+(C5=0)*0.0001,"Perto","Fora")),IF(B5&gt;=C5,"No alvo",IF(B5&gt;=C5*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B5="",C5=""),"Informativo",IF(D5="Menor é melhor",IF(B5&lt;C5,"No alvo",IF(B5&lt;=C5*1.1+(C5=0)*0.0001,"Perto","Fora")),IF(B5&gt;C5,"No alvo",IF(B5&gt;=C5*0.9,"Perto","Fora"))))</f>
         <v>No alvo</v>
       </c>
     </row>
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="F6" s="19" t="str">
-        <f>IF(OR(B6="",C6=""),"Informativo",IF(D6="Menor é melhor",IF(B6&lt;=C6,"No alvo",IF(B6&lt;=C6*1.1+(C6=0)*0.0001,"Perto","Fora")),IF(B6&gt;=C6,"No alvo",IF(B6&gt;=C6*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B6="",C6=""),"Informativo",IF(D6="Menor é melhor",IF(B6&lt;C6,"No alvo",IF(B6&lt;=C6*1.1+(C6=0)*0.0001,"Perto","Fora")),IF(B6&gt;C6,"No alvo",IF(B6&gt;=C6*0.9,"Perto","Fora"))))</f>
         <v>Informativo</v>
       </c>
     </row>
@@ -2516,7 +2516,7 @@
         </is>
       </c>
       <c r="F7" s="19" t="str">
-        <f>IF(OR(B7="",C7=""),"Informativo",IF(D7="Menor é melhor",IF(B7&lt;=C7,"No alvo",IF(B7&lt;=C7*1.1+(C7=0)*0.0001,"Perto","Fora")),IF(B7&gt;=C7,"No alvo",IF(B7&gt;=C7*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B7="",C7=""),"Informativo",IF(D7="Menor é melhor",IF(B7&lt;C7,"No alvo",IF(B7&lt;=C7*1.1+(C7=0)*0.0001,"Perto","Fora")),IF(B7&gt;C7,"No alvo",IF(B7&gt;=C7*0.9,"Perto","Fora"))))</f>
         <v>Informativo</v>
       </c>
     </row>
@@ -2543,7 +2543,7 @@
         </is>
       </c>
       <c r="F8" s="19" t="str">
-        <f>IF(OR(B8="",C8=""),"Informativo",IF(D8="Menor é melhor",IF(B8&lt;=C8,"No alvo",IF(B8&lt;=C8*1.1+(C8=0)*0.0001,"Perto","Fora")),IF(B8&gt;=C8,"No alvo",IF(B8&gt;=C8*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B8="",C8=""),"Informativo",IF(D8="Menor é melhor",IF(B8&lt;C8,"No alvo",IF(B8&lt;=C8*1.1+(C8=0)*0.0001,"Perto","Fora")),IF(B8&gt;C8,"No alvo",IF(B8&gt;=C8*0.9,"Perto","Fora"))))</f>
         <v>No alvo</v>
       </c>
     </row>
@@ -2570,8 +2570,8 @@
         </is>
       </c>
       <c r="F9" s="19" t="str">
-        <f>IF(OR(B9="",C9=""),"Informativo",IF(D9="Menor é melhor",IF(B9&lt;=C9,"No alvo",IF(B9&lt;=C9*1.1+(C9=0)*0.0001,"Perto","Fora")),IF(B9&gt;=C9,"No alvo",IF(B9&gt;=C9*0.9,"Perto","Fora"))))</f>
-        <v>No alvo</v>
+        <f>IF(OR(B9="",C9=""),"Informativo",IF(D9="Menor é melhor",IF(B9&lt;C9,"No alvo",IF(B9&lt;=C9*1.1+(C9=0)*0.0001,"Perto","Fora")),IF(B9&gt;C9,"No alvo",IF(B9&gt;=C9*0.9,"Perto","Fora"))))</f>
+        <v>Perto</v>
       </c>
     </row>
     <row r="10">
@@ -2591,7 +2591,7 @@
         </is>
       </c>
       <c r="F10" s="19" t="str">
-        <f>IF(OR(B10="",C10=""),"Informativo",IF(D10="Menor é melhor",IF(B10&lt;=C10,"No alvo",IF(B10&lt;=C10*1.1+(C10=0)*0.0001,"Perto","Fora")),IF(B10&gt;=C10,"No alvo",IF(B10&gt;=C10*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B10="",C10=""),"Informativo",IF(D10="Menor é melhor",IF(B10&lt;C10,"No alvo",IF(B10&lt;=C10*1.1+(C10=0)*0.0001,"Perto","Fora")),IF(B10&gt;C10,"No alvo",IF(B10&gt;=C10*0.9,"Perto","Fora"))))</f>
         <v>Informativo</v>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         </is>
       </c>
       <c r="F11" s="19" t="str">
-        <f>IF(OR(B11="",C11=""),"Informativo",IF(D11="Menor é melhor",IF(B11&lt;=C11,"No alvo",IF(B11&lt;=C11*1.1+(C11=0)*0.0001,"Perto","Fora")),IF(B11&gt;=C11,"No alvo",IF(B11&gt;=C11*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B11="",C11=""),"Informativo",IF(D11="Menor é melhor",IF(B11&lt;C11,"No alvo",IF(B11&lt;=C11*1.1+(C11=0)*0.0001,"Perto","Fora")),IF(B11&gt;C11,"No alvo",IF(B11&gt;=C11*0.9,"Perto","Fora"))))</f>
         <v>Informativo</v>
       </c>
     </row>
@@ -2634,7 +2634,7 @@
         </is>
       </c>
       <c r="F12" s="19" t="str">
-        <f>IF(OR(B12="",C12=""),"Informativo",IF(D12="Menor é melhor",IF(B12&lt;=C12,"No alvo",IF(B12&lt;=C12*1.1+(C12=0)*0.0001,"Perto","Fora")),IF(B12&gt;=C12,"No alvo",IF(B12&gt;=C12*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B12="",C12=""),"Informativo",IF(D12="Menor é melhor",IF(B12&lt;C12,"No alvo",IF(B12&lt;=C12*1.1+(C12=0)*0.0001,"Perto","Fora")),IF(B12&gt;C12,"No alvo",IF(B12&gt;=C12*0.9,"Perto","Fora"))))</f>
         <v>Informativo</v>
       </c>
     </row>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="F13" s="19" t="str">
-        <f>IF(OR(B13="",C13=""),"Informativo",IF(D13="Menor é melhor",IF(B13&lt;=C13,"No alvo",IF(B13&lt;=C13*1.1+(C13=0)*0.0001,"Perto","Fora")),IF(B13&gt;=C13,"No alvo",IF(B13&gt;=C13*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B13="",C13=""),"Informativo",IF(D13="Menor é melhor",IF(B13&lt;C13,"No alvo",IF(B13&lt;=C13*1.1+(C13=0)*0.0001,"Perto","Fora")),IF(B13&gt;C13,"No alvo",IF(B13&gt;=C13*0.9,"Perto","Fora"))))</f>
         <v>Informativo</v>
       </c>
     </row>
@@ -2682,7 +2682,7 @@
         </is>
       </c>
       <c r="F14" s="19" t="str">
-        <f>IF(OR(B14="",C14=""),"Informativo",IF(D14="Menor é melhor",IF(B14&lt;=C14,"No alvo",IF(B14&lt;=C14*1.1+(C14=0)*0.0001,"Perto","Fora")),IF(B14&gt;=C14,"No alvo",IF(B14&gt;=C14*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B14="",C14=""),"Informativo",IF(D14="Menor é melhor",IF(B14&lt;C14,"No alvo",IF(B14&lt;=C14*1.1+(C14=0)*0.0001,"Perto","Fora")),IF(B14&gt;C14,"No alvo",IF(B14&gt;=C14*0.9,"Perto","Fora"))))</f>
         <v>Fora</v>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="F15" s="19" t="str">
-        <f>IF(OR(B15="",C15=""),"Informativo",IF(D15="Menor é melhor",IF(B15&lt;=C15,"No alvo",IF(B15&lt;=C15*1.1+(C15=0)*0.0001,"Perto","Fora")),IF(B15&gt;=C15,"No alvo",IF(B15&gt;=C15*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B15="",C15=""),"Informativo",IF(D15="Menor é melhor",IF(B15&lt;C15,"No alvo",IF(B15&lt;=C15*1.1+(C15=0)*0.0001,"Perto","Fora")),IF(B15&gt;C15,"No alvo",IF(B15&gt;=C15*0.9,"Perto","Fora"))))</f>
         <v>Fora</v>
       </c>
     </row>
@@ -2736,7 +2736,7 @@
         </is>
       </c>
       <c r="F16" s="19" t="str">
-        <f>IF(OR(B16="",C16=""),"Informativo",IF(D16="Menor é melhor",IF(B16&lt;=C16,"No alvo",IF(B16&lt;=C16*1.1+(C16=0)*0.0001,"Perto","Fora")),IF(B16&gt;=C16,"No alvo",IF(B16&gt;=C16*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B16="",C16=""),"Informativo",IF(D16="Menor é melhor",IF(B16&lt;C16,"No alvo",IF(B16&lt;=C16*1.1+(C16=0)*0.0001,"Perto","Fora")),IF(B16&gt;C16,"No alvo",IF(B16&gt;=C16*0.9,"Perto","Fora"))))</f>
         <v>No alvo</v>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
         </is>
       </c>
       <c r="F17" s="19" t="str">
-        <f>IF(OR(B17="",C17=""),"Informativo",IF(D17="Menor é melhor",IF(B17&lt;=C17,"No alvo",IF(B17&lt;=C17*1.1+(C17=0)*0.0001,"Perto","Fora")),IF(B17&gt;=C17,"No alvo",IF(B17&gt;=C17*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B17="",C17=""),"Informativo",IF(D17="Menor é melhor",IF(B17&lt;C17,"No alvo",IF(B17&lt;=C17*1.1+(C17=0)*0.0001,"Perto","Fora")),IF(B17&gt;C17,"No alvo",IF(B17&gt;=C17*0.9,"Perto","Fora"))))</f>
         <v>Fora</v>
       </c>
     </row>
@@ -2784,7 +2784,7 @@
         </is>
       </c>
       <c r="F18" s="19" t="str">
-        <f>IF(OR(B18="",C18=""),"Informativo",IF(D18="Menor é melhor",IF(B18&lt;=C18,"No alvo",IF(B18&lt;=C18*1.1+(C18=0)*0.0001,"Perto","Fora")),IF(B18&gt;=C18,"No alvo",IF(B18&gt;=C18*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B18="",C18=""),"Informativo",IF(D18="Menor é melhor",IF(B18&lt;C18,"No alvo",IF(B18&lt;=C18*1.1+(C18=0)*0.0001,"Perto","Fora")),IF(B18&gt;C18,"No alvo",IF(B18&gt;=C18*0.9,"Perto","Fora"))))</f>
         <v>Informativo</v>
       </c>
     </row>
@@ -2805,14 +2805,14 @@
         </is>
       </c>
       <c r="F19" s="19" t="str">
-        <f>IF(OR(B19="",C19=""),"Informativo",IF(D19="Menor é melhor",IF(B19&lt;=C19,"No alvo",IF(B19&lt;=C19*1.1+(C19=0)*0.0001,"Perto","Fora")),IF(B19&gt;=C19,"No alvo",IF(B19&gt;=C19*0.9,"Perto","Fora"))))</f>
+        <f>IF(OR(B19="",C19=""),"Informativo",IF(D19="Menor é melhor",IF(B19&lt;C19,"No alvo",IF(B19&lt;=C19*1.1+(C19=0)*0.0001,"Perto","Fora")),IF(B19&gt;C19,"No alvo",IF(B19&gt;=C19*0.9,"Perto","Fora"))))</f>
         <v>Informativo</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>Linha sem limite fica "Informativo". "Perto" é até 10% do limite. Inadimplência = vencido ÷ (pago + vencido), a mesma conta da planilha 14. Convênio a receber é o que foi enviado e ainda está no prazo: informativo; o problema é o atrasado. Orçamentos em aberto também são informativos: pouco orçamento pendente pode ser bom (fechou tudo) ou ruim (a recepção parou de apresentar) — quem diz é a taxa de aprovação da planilha 15, não o valor parado. Os valores desta sexta valem para o mês escolhido em Config; no fim do mês, copie a coluna B para a linha do mês em Histórico.</t>
+          <t>Linha sem limite fica "Informativo". "Perto" é o limite exato ou até 10% além dele. Inadimplência = vencido ÷ (pago + vencido), a mesma conta da planilha 14. Convênio a receber é o que foi enviado e ainda está no prazo: informativo; o problema é o atrasado. Orçamentos em aberto também são informativos: pouco orçamento pendente pode ser bom (fechou tudo) ou ruim (a recepção parou de apresentar) — quem diz é a taxa de aprovação da planilha 15, não o valor parado. Os valores desta sexta valem para o mês escolhido em Config; no fim do mês, copie a coluna B para a linha do mês em Histórico.</t>
         </is>
       </c>
     </row>

</xml_diff>